<commit_message>
Add evolving knowledge ingestion, PDF replacement and evaluation tooling
</commit_message>
<xml_diff>
--- a/data/raw/conversations_source_01.xlsx
+++ b/data/raw/conversations_source_01.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tickets" sheetId="1" r:id="Rb209e658286c4825"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" r:id="R8dfeda03a8504185"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="3" r:id="Rdaba4bc5823c42d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counts" sheetId="4" r:id="Rf3d3519a52514cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tickets" sheetId="1" r:id="R60ca0dadddbd4da7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" r:id="Rc4fc4a6c2ac64cfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="3" r:id="R9b41e1fde3704cdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counts" sheetId="4" r:id="Rffa0d2bfd0344cdf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -46,13 +46,7 @@
     </x:fill>
   </x:fills>
   <x:borders count="1">
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
+    <x:border/>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -399,28 +393,34 @@
         <x:v>Fiber Broadband &amp; Gateway</x:v>
       </x:c>
       <x:c r="F2" s="3" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
         <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
-        <x:v>Seven minutes of steady service, a brief drop, then seven minutes again. Our café terminal log matches the WAN renewal events almost exactly.</x:v>
+        <x:v>Our fibre gateway restarts at the same time every afternoon. Its settings show an automatic reboot schedule that we did not intend to enable. I am frustrated with this situation.</x:v>
       </x:c>
       <x:c r="I2" s="3" t="str">
-        <x:v>Customer: Seven minutes of steady service, a brief drop, then seven minutes again. Our café terminal log matches the WAN renewal events almost exactly.
-Agent: Can access support inspect the renewal exchange rather than asking you to reboot?
-Customer: They found inconsistent renewal responses; the café's terminal stopped dropping after the controlled repair.
-Agent: Repairing the access DHCP renewal handling stopped the café's periodic WAN interruptions.</x:v>
+        <x:v>Customer: Our fibre gateway restarts at the same time every afternoon. Its settings show an automatic reboot schedule that we did not intend to enable. I am frustrated with this situation.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify the configured scheduled-reboot policy.
+2. Match reboot events to reported interruptions.
+3. Disable the unintended reboot schedule with customer consent.
+4. Verify normal operation at the formerly scheduled time.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J2" s="3" t="str">
-        <x:v>1. Compare WAN renewal timestamps with drop logs.
-2. Inspect the access DHCP renewal exchange.
-3. Repair the confirmed DHCP renewal handling through network operations.
-4. Verify uninterrupted connectivity over multiple lease renewals.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify the configured scheduled-reboot policy.
+2. Match reboot events to reported interruptions.
+3. Disable the unintended reboot schedule with customer consent.
+4. Verify normal operation at the formerly scheduled time.</x:v>
       </x:c>
       <x:c r="K2" s="3" t="str">
-        <x:v>Repairing the access DHCP renewal handling stopped the café's periodic WAN interruptions.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L2" s="3" t="str">
         <x:v>approved for historical</x:v>
@@ -447,7 +447,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
         <x:v>School pickup time isn't the cause after all: the gateway has an automatic reboot set for 15:15. I didn't knowingly schedule it.</x:v>
@@ -492,7 +492,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>Annoyed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
         <x:v>Guests return from dinner to a connection that needs waking up. It behaves once traffic starts, but the access session closes after inactivity.</x:v>
@@ -582,7 +582,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
         <x:v>Living under the flight path seems to matter: wireless vanishes during logged radar events, although ethernet never blinks.</x:v>
@@ -672,7 +672,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
         <x:v>Primary fiber looks healthy, backup looks healthy, yet the managed router keeps bouncing between them and breaking sessions. That cannot be sensible.</x:v>
@@ -717,7 +717,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G9" s="3" t="str">
-        <x:v>Annoyed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H9" s="3" t="str">
         <x:v>A colleague plugged in a second gateway and now ours keeps getting signed out. Support says this account permits one active access session.</x:v>
@@ -762,7 +762,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
-        <x:v>Disappointed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H10" s="3" t="str">
         <x:v>EEE sleep on the new office switch appears to cut its link to the fiber gateway whenever traffic goes quiet. Fiber itself stays registered.</x:v>
@@ -804,28 +804,34 @@
         <x:v>Fiber Broadband &amp; Gateway</x:v>
       </x:c>
       <x:c r="F11" s="3" t="str">
-        <x:v>Low</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H11" s="3" t="str">
-        <x:v>Seeing twelve megabytes a second made me think a hundred-megabit subscription was broken. A normal speed test disagrees with that worry.</x:v>
+        <x:v>The guest Wi-Fi is much slower than the staff network. An old bandwidth limit is still configured on the guest SSID. I am frustrated with this situation.</x:v>
       </x:c>
       <x:c r="I11" s="3" t="str">
-        <x:v>Customer: Seeing twelve megabytes a second made me think a hundred-megabit subscription was broken. A normal speed test disagrees with that worry.
-Agent: Shall we compare the application's byte-based display with the plan's bit-based rate?
-Customer: The units explain it and the supported test confirms normal service performance.
-Agent: Explaining MB/s versus Mbps reconciled the download display with normal service performance.</x:v>
+        <x:v>Customer: The guest Wi-Fi is much slower than the staff network. An old bandwidth limit is still configured on the guest SSID. I am frustrated with this situation.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Compare guest and staff performance under controlled conditions.
+2. Inspect per-SSID bandwidth settings.
+3. Correct the unintended guest-network cap with administrator consent.
+4. Verify guest access while preserving network separation.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J11" s="3" t="str">
-        <x:v>1. Identify the units used by the application and subscribed plan.
-2. Explain the eight-bit-to-one-byte conversion and protocol overhead.
-3. Run a controlled supported speed test.
-4. Confirm whether measured service performance matches the plan.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Compare guest and staff performance under controlled conditions.
+2. Inspect per-SSID bandwidth settings.
+3. Correct the unintended guest-network cap with administrator consent.
+4. Verify guest access while preserving network separation.</x:v>
       </x:c>
       <x:c r="K11" s="3" t="str">
-        <x:v>Explaining MB/s versus Mbps reconciled the download display with normal service performance.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L11" s="3" t="str">
         <x:v>approved for historical</x:v>
@@ -942,7 +948,7 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="G14" s="3" t="str">
-        <x:v>Annoyed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H14" s="3" t="str">
         <x:v>Plain browser: quick. Browser full of optional add-ons: painfully slow. Everything else on the fiber service is fine, so please start there.</x:v>
@@ -987,7 +993,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G15" s="3" t="str">
-        <x:v>Disappointed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H15" s="3" t="str">
         <x:v>Our supplier's portal is the only destination dragging from this connection. Network measurements point to the interconnection, not the office LAN.</x:v>
@@ -1077,7 +1083,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G17" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H17" s="3" t="str">
         <x:v>Downloads crawl on a crowded Wi-Fi channel in this apartment block, but a direct ethernet test is quick. Can we assess airtime before changing my plan?</x:v>
@@ -1122,7 +1128,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G18" s="3" t="str">
-        <x:v>Disappointed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H18" s="3" t="str">
         <x:v>Our fiber speed is restricted by a stale protective policer left after an incident. Operations says the incident is cleared but the policy is still attached.</x:v>
@@ -1257,25 +1263,31 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G21" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H21" s="3" t="str">
-        <x:v>Our managed site tunnel stopped at the certificate expiry timestamp. Warehouse access is down; local cabling and power are normal.</x:v>
+        <x:v>Our office broadband is completely offline. The gateway cannot obtain a new WAN address, and the diagnostics report subscriber address-pool exhaustion. I am frustrated with this situation.</x:v>
       </x:c>
       <x:c r="I21" s="3" t="str">
-        <x:v>Customer: Our managed site tunnel stopped at the certificate expiry timestamp. Warehouse access is down; local cabling and power are normal.
-Agent: Can the controlled certificate process renew the verified gateway identity?
-Customer: The authorised renewal completed and the tunnel now carries warehouse traffic again.
-Agent: Renewing the managed gateway certificate restored the warehouse access tunnel.</x:v>
+        <x:v>Customer: Our office broadband is completely offline. The gateway cannot obtain a new WAN address, and the diagnostics report subscriber address-pool exhaustion. I am frustrated with this situation.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Check WAN address-allocation failures and access-service alarms.
+2. Confirm subscriber pool exhaustion through network operations.
+3. Restore authorised pool capacity or allocation handling.
+4. Verify new sessions receive valid WAN addresses.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J21" s="3" t="str">
-        <x:v>1. Verify managed-tunnel status and certificate validity through approved systems.
-2. Confirm the authorised identity of the gateway.
-3. Renew and deploy the certificate using the controlled certificate lifecycle.
-4. Verify tunnel establishment and site connectivity.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Check WAN address-allocation failures and access-service alarms.
+2. Confirm subscriber pool exhaustion through network operations.
+3. Restore authorised pool capacity or allocation handling.
+4. Verify new sessions receive valid WAN addresses.</x:v>
       </x:c>
       <x:c r="K21" s="3" t="str">
-        <x:v>Renewing the managed gateway certificate restored the warehouse access tunnel.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L21" s="3" t="str">
         <x:v>approved for historical</x:v>
@@ -1302,7 +1314,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G22" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H22" s="3" t="str">
         <x:v>Followed forum advice to disable IPv6, then discovered this service carries IPv4 through DS-Lite. We have managed to switch off its transport.</x:v>
@@ -1344,10 +1356,10 @@
         <x:v>Fiber Broadband &amp; Gateway</x:v>
       </x:c>
       <x:c r="F23" s="3" t="str">
-        <x:v>Critical</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G23" s="3" t="str">
-        <x:v>Panicked</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H23" s="3" t="str">
         <x:v>A route withdrawal has taken our remote booking operation fully offline. Circuit is up, backup unavailable, and customers cannot be served.</x:v>
@@ -1392,7 +1404,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G24" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H24" s="3" t="str">
         <x:v>Security mitigation is active but legitimate traffic to our office is being dropped by the mitigation routing. Our security contact can coordinate the correction.</x:v>
@@ -1437,7 +1449,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G25" s="3" t="str">
-        <x:v>Disappointed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H25" s="3" t="str">
         <x:v>Healthy optical readings, zero internet traffic after handover. The wholesale records list a different VLAN from the one actually configured.</x:v>
@@ -1527,7 +1539,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G27" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H27" s="3" t="str">
         <x:v>The static address looks right but its subnet mask doesn't match the provider sheet. Even the WAN next hop is unreachable at this branch.</x:v>
@@ -1572,7 +1584,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G28" s="3" t="str">
-        <x:v>Annoyed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
         <x:v>Bridge mode is enabled and there's no subscriber dialler configured on our own firewall. The gateway isn't supposed to start that session anymore.</x:v>
@@ -1617,7 +1629,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G29" s="3" t="str">
-        <x:v>Panicked</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H29" s="3" t="str">
         <x:v>Roof leak reached the gateway shelf. Unit is off, nobody will open it, and we need qualified replacement rather than drying instructions.</x:v>
@@ -1662,25 +1674,31 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G30" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H30" s="3" t="str">
-        <x:v>The backup battery beside our ONT has visibly deformed. We have cleared the immediate area and need the equipment safety team to handle it.</x:v>
+        <x:v>A water leak reached our broadband gateway. We have kept the damaged unit out of use and will not open it. Please arrange the approved assessment. I am frustrated with this situation.</x:v>
       </x:c>
       <x:c r="I30" s="3" t="str">
-        <x:v>Customer: The backup battery beside our ONT has visibly deformed. We have cleared the immediate area and need the equipment safety team to handle it.
-Agent: Can it remain undisturbed until qualified personnel follow the approved safety procedure?
-Customer: Qualified personnel isolated and replaced the damaged battery; safe operation was verified.
-Agent: Qualified replacement of the damaged ONT backup battery restored safe equipment operation.</x:v>
+        <x:v>Customer: A water leak reached our broadband gateway. We have kept the damaged unit out of use and will not open it. Please arrange the approved assessment. I am frustrated with this situation.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Keep water-damaged equipment out of use and avoid unsafe handling.
+2. Record safe observations without opening the enclosure.
+3. Arrange authorised assessment and replacement according to eligibility.
+4. Verify service on the safely installed replacement.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J30" s="3" t="str">
-        <x:v>1. Advise avoiding contact or tampering with the visibly damaged battery.
-2. Escalate through the approved equipment safety process.
-3. Have qualified personnel isolate and replace the battery as appropriate.
-4. Verify safe equipment operation after authorised work.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Keep water-damaged equipment out of use and avoid unsafe handling.
+2. Record safe observations without opening the enclosure.
+3. Arrange authorised assessment and replacement according to eligibility.
+4. Verify service on the safely installed replacement.</x:v>
       </x:c>
       <x:c r="K30" s="3" t="str">
-        <x:v>Qualified replacement of the damaged ONT backup battery restored safe equipment operation.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L30" s="3" t="str">
         <x:v>approved for historical</x:v>
@@ -1707,7 +1725,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G31" s="3" t="str">
-        <x:v>Disappointed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H31" s="3" t="str">
         <x:v>A shelf collapsed and broke the router's external aerial. Wired service survived; wireless reception didn't. No amount of password changing will repair that.</x:v>
@@ -1842,7 +1860,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G34" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H34" s="3" t="str">
         <x:v>The gateway sits in an approved external cabinet, but a corroded Ethernet receptacle is now losing contact. A field inspection has confirmed the port damage.</x:v>
@@ -1887,7 +1905,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G35" s="3" t="str">
-        <x:v>Annoyed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H35" s="3" t="str">
         <x:v>Fiber still works, but our gateway's USB backup-modem socket is cracked and cannot hold a connection. The approved modem is fine on another unit.</x:v>
@@ -1932,7 +1950,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G36" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H36" s="3" t="str">
         <x:v>Fan-failure alarm on the managed edge router; still online, but operations needs controlled maintenance before overheating occurs.</x:v>
@@ -2067,7 +2085,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G39" s="3" t="str">
-        <x:v>Annoyed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H39" s="3" t="str">
         <x:v>Depot receipt proves the rented gateway was returned, yet a non-return fee remains. The serial number on the receipt matches the service record.</x:v>
@@ -2202,7 +2220,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G42" s="3" t="str">
-        <x:v>Disappointed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H42" s="3" t="str">
         <x:v>Your team approved an outage adjustment under an existing reference, but the ledger never received it. Please trace that approval rather than reopen eligibility.</x:v>
@@ -2382,25 +2400,31 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G46" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H46" s="3" t="str">
-        <x:v>Near the border, the phone registered on the neighbouring country's network without us travelling there. I'd like the roaming records reviewed under the actual policy.</x:v>
+        <x:v>My telecom invoice has been paid twice. Two settled payment references appear in the account ledger for the same bill, and I want the duplicate reconciled. I am frustrated with this situation.</x:v>
       </x:c>
       <x:c r="I46" s="3" t="str">
-        <x:v>Customer: Near the border, the phone registered on the neighbouring country's network without us travelling there. I'd like the roaming records reviewed under the actual policy.
-Agent: Do the records confirm border registration, and has an adjustment been expressly authorised?
-Customer: Both are confirmed; the approved adjustment was processed and supported network-selection precautions explained.
-Agent: An authorised border-roaming adjustment resolved the disputed charges and clarified network-selection precautions.</x:v>
+        <x:v>Customer: My telecom invoice has been paid twice. Two settled payment references appear in the account ledger for the same bill, and I want the duplicate reconciled. I am frustrated with this situation.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify identity through the approved billing channel.
+2. Reconcile both settled payment references against the invoice.
+3. Obtain authorised approval for the duplicate-payment refund or agreed balance treatment.
+4. Confirm the processed adjustment and remaining balance.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J46" s="3" t="str">
-        <x:v>1. Inspect roaming network and usage records against applicable plan terms.
-2. Explain border-network registration and supported manual selection precautions.
-3. Process only an explicitly approved adjustment.
-4. Confirm the corrected bill and supported prevention settings.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify identity through the approved billing channel.
+2. Reconcile both settled payment references against the invoice.
+3. Obtain authorised approval for the duplicate-payment refund or agreed balance treatment.
+4. Confirm the processed adjustment and remaining balance.</x:v>
       </x:c>
       <x:c r="K46" s="3" t="str">
-        <x:v>An authorised border-roaming adjustment resolved the disputed charges and clarified network-selection precautions.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L46" s="3" t="str">
         <x:v>approved for historical</x:v>
@@ -2517,7 +2541,7 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="G49" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H49" s="3" t="str">
         <x:v>Four colleagues will join the company data pool. Their numbers must stay intact and I'd like each eligibility checked first.</x:v>
@@ -2607,25 +2631,31 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="G51" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H51" s="3" t="str">
-        <x:v>Leaving the apartment empty for a while. Does this fiber subscription permit a temporary pause, and what are the exact billing and return-to-service conditions?</x:v>
+        <x:v>We need broadband for a second business location with its own invoice. This is a separate service request, not an upgrade to the existing branch connection. I am frustrated with this situation.</x:v>
       </x:c>
       <x:c r="I51" s="3" t="str">
-        <x:v>Customer: Leaving the apartment empty for a while. Does this fiber subscription permit a temporary pause, and what are the exact billing and return-to-service conditions?
-Agent: Can we review the published eligibility rather than assume a pause is available?
-Customer: The pause is eligible; I accepted its documented dates and restoration conditions.
-Agent: An authorised temporary service pause was scheduled under the verified subscription terms.</x:v>
+        <x:v>Customer: We need broadband for a second business location with its own invoice. This is a separate service request, not an upgrade to the existing branch connection. I am frustrated with this situation.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify authorised business contact and new-site eligibility.
+2. Distinguish a second service order from modifying the existing line.
+3. Present documented separate-billing and contract terms.
+4. Process the accepted eligible new-site order and confirm both service records.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J51" s="3" t="str">
-        <x:v>1. Verify account authority and temporary-pause eligibility.
-2. Explain documented billing and restoration conditions.
-3. Obtain consent for the agreed pause interval.
-4. Record the authorised pause and confirm its effective dates.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify authorised business contact and new-site eligibility.
+2. Distinguish a second service order from modifying the existing line.
+3. Present documented separate-billing and contract terms.
+4. Process the accepted eligible new-site order and confirm both service records.</x:v>
       </x:c>
       <x:c r="K51" s="3" t="str">
-        <x:v>An authorised temporary service pause was scheduled under the verified subscription terms.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L51" s="3" t="str">
         <x:v>approved for historical</x:v>
@@ -2697,7 +2727,7 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="G53" s="3" t="str">
-        <x:v>Annoyed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H53" s="3" t="str">
         <x:v>Order preview starts the mobile tariff today; my intended date is the eligible next billing boundary. Please correct the preview before taking consent.</x:v>
@@ -2835,22 +2865,28 @@
         <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H56" s="3" t="str">
-        <x:v>Passenger calls repeatedly cut at the same cell boundary on the ring road. We recorded times safely; fixed-location service elsewhere is normal.</x:v>
+        <x:v>Mobile reception became weaker in one business-park sector after antenna work. Compatible handsets show the same local pattern, but coverage elsewhere is normal. I am frustrated with this situation.</x:v>
       </x:c>
       <x:c r="I56" s="3" t="str">
-        <x:v>Customer: Passenger calls repeatedly cut at the same cell boundary on the ring road. We recorded times safely; fixed-location service elsewhere is normal.
-Agent: Can radio engineering compare those observations with the handover traces?
-Customer: They confirmed a handover configuration fault and approved testing passes after correction.
-Agent: A radio handover configuration correction improved call continuity between the affected cells.</x:v>
+        <x:v>Customer: Mobile reception became weaker in one business-park sector after antenna work. Compatible handsets show the same local pattern, but coverage elsewhere is normal. I am frustrated with this situation.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Collect location-specific supported-device observations.
+2. Compare sector alarms and authorised post-work measurements.
+3. Correct the verified sector configuration through radio engineering.
+4. Retest coverage in the affected area.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J56" s="3" t="str">
-        <x:v>1. Collect safe passenger-observed times and affected locations.
-2. Compare radio handover traces and service incidents.
-3. Correct the confirmed cell handover configuration through radio engineering.
-4. Verify mobility calls through approved testing.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Collect location-specific supported-device observations.
+2. Compare sector alarms and authorised post-work measurements.
+3. Correct the verified sector configuration through radio engineering.
+4. Retest coverage in the affected area.</x:v>
       </x:c>
       <x:c r="K56" s="3" t="str">
-        <x:v>A radio handover configuration correction improved call continuity between the affected cells.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L56" s="3" t="str">
         <x:v>approved for historical</x:v>
@@ -2922,7 +2958,7 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="G58" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H58" s="3" t="str">
         <x:v>That decorative metal cover looked good until it wrecked reception. Bare handset behaves normally at exactly the same spot.</x:v>
@@ -2967,7 +3003,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G59" s="3" t="str">
-        <x:v>Annoyed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H59" s="3" t="str">
         <x:v>Forced 5G-only in a hidden menu, then lost usable service in a location with supported 4G. I realise this may be self-inflicted.</x:v>
@@ -3012,7 +3048,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G60" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H60" s="3" t="str">
         <x:v>Warehouse corner has a radio disturbance pattern, not just low signal. Please assess interference instead of telling us to install an unapproved booster.</x:v>
@@ -3057,7 +3093,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G61" s="3" t="str">
-        <x:v>Disappointed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H61" s="3" t="str">
         <x:v>Bought an imported handset and discovered its band support may not match the network. A compatible phone on the same SIM is fine.</x:v>
@@ -3237,7 +3273,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G65" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H65" s="3" t="str">
         <x:v>Serial on the new SIM belongs to another pending order in the activation screen. We stopped before activating anything against the wrong subscription.</x:v>
@@ -3282,7 +3318,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G66" s="3" t="str">
-        <x:v>Disappointed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H66" s="3" t="str">
         <x:v>eSIM profile is valid, but the handset is locked to its original carrier. I need the legitimate eligibility route, not endless replacement QR codes.</x:v>
@@ -3327,7 +3363,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G67" s="3" t="str">
-        <x:v>Panicked</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H67" s="3" t="str">
         <x:v>We cancelled the donor line too early and the port request is blocked. Please check the actual recovery eligibility rather than guaranteeing the number can be saved.</x:v>
@@ -3372,7 +3408,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G68" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H68" s="3" t="str">
         <x:v>Stopped entering PINs when the SIM requested PUK. Account owner is available for secure verification; please use the official unblock process.</x:v>
@@ -3417,7 +3453,7 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="G69" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H69" s="3" t="str">
         <x:v>Two active profiles, wrong default for outgoing texts. The activation message goes from the personal number instead of the new work line.</x:v>
@@ -3462,25 +3498,31 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G70" s="3" t="str">
-        <x:v>Panicked</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H70" s="3" t="str">
-        <x:v>Phone disappeared with the active work SIM inside. We need the verified loss process to restrict it and arrange the authorised replacement.</x:v>
+        <x:v>My replacement SIM cannot be activated and I have no mobile calling service. Its serial is assigned to a different pending order in the activation record. I am frustrated with this situation.</x:v>
       </x:c>
       <x:c r="I70" s="3" t="str">
-        <x:v>Customer: Phone disappeared with the active work SIM inside. We need the verified loss process to restrict it and arrange the authorised replacement.
-Agent: Can secure ownership verification establish the affected line and approve the loss-response actions?
-Customer: It did; the old profile was barred and retired, and the authorised replacement has working service.
-Agent: An authorised lost-SIM restriction and replacement restored service while disabling the lost profile.</x:v>
+        <x:v>Customer: My replacement SIM cannot be activated and I have no mobile calling service. Its serial is assigned to a different pending order in the activation record. I am frustrated with this situation.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify identity and authorised order references securely.
+2. Compare SIM serial assignment with the intended order.
+3. Correct the verified assignment through activation operations.
+4. Activate the eligible SIM and verify service.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J70" s="3" t="str">
-        <x:v>1. Verify ownership through the approved loss-response channel.
-2. Apply authorised restrictions to the lost SIM.
-3. Fulfil the verified replacement and retire the lost profile.
-4. Verify service on the replacement device.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify identity and authorised order references securely.
+2. Compare SIM serial assignment with the intended order.
+3. Correct the verified assignment through activation operations.
+4. Activate the eligible SIM and verify service.</x:v>
       </x:c>
       <x:c r="K70" s="3" t="str">
-        <x:v>An authorised lost-SIM restriction and replacement restored service while disabling the lost profile.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L70" s="3" t="str">
         <x:v>approved for historical</x:v>
@@ -3507,7 +3549,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G71" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H71" s="3" t="str">
         <x:v>Most of our business SIM order is active; two jobs failed despite correct serial assignments. Please inspect those jobs before submitting duplicates.</x:v>
@@ -3597,7 +3639,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G73" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H73" s="3" t="str">
         <x:v>Handset won't accept another eSIM because its stored-profile limit is reached. There's an obsolete inactive one, but I want to avoid deleting an active line.</x:v>
@@ -3687,7 +3729,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G75" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H75" s="3" t="str">
         <x:v>Protected frontage needs a lawful entry route for the connection. Please arrange planning review before anyone drills through it.</x:v>
@@ -3732,7 +3774,7 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="G76" s="3" t="str">
-        <x:v>Annoyed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H76" s="3" t="str">
         <x:v>The office calendar says local morning; dispatch has the same clock time in a different timezone. Could we reconcile the confirmation before the visit?</x:v>
@@ -3777,7 +3819,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G77" s="3" t="str">
-        <x:v>Disappointed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H77" s="3" t="str">
         <x:v>Commissioning stopped because the supplied gateway model cannot deliver the ordered handoff. Sending the same model again would waste another appointment.</x:v>
@@ -3867,7 +3909,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G79" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H79" s="3" t="str">
         <x:v>The field order requires splicing skills that the assigned customer-equipment crew doesn't have. Please align qualifications with the work.</x:v>
@@ -3954,28 +3996,34 @@
         <x:v>Home Installation / Technical Visit</x:v>
       </x:c>
       <x:c r="F81" s="3" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="G81" s="3" t="str">
-        <x:v>Disappointed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H81" s="3" t="str">
-        <x:v>Outdoor appointment was stopped by the authorised weather restriction. That's understood; we'd like a real available slot once safe field work resumes.</x:v>
+        <x:v>The apartment fibre installation needs written building-association permission for the proposed cable route. That approval has not been obtained yet. I am frustrated with this situation.</x:v>
       </x:c>
       <x:c r="I81" s="3" t="str">
-        <x:v>Customer: Outdoor appointment was stopped by the authorised weather restriction. That's understood; we'd like a real available slot once safe field work resumes.
-Agent: Has dispatch confirmed a permitted replacement slot after restrictions lift?
-Customer: Yes; we accepted the confirmed slot and the safe installation completed.
-Agent: Rebooking after the authorised weather restriction lifted completed the outdoor installation safely.</x:v>
+        <x:v>Customer: The apartment fibre installation needs written building-association permission for the proposed cable route. That approval has not been obtained yet. I am frustrated with this situation.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify the recorded building permission requirement.
+2. Coordinate an approved route proposal with authorised building contacts.
+3. Obtain the necessary permission before scheduling installation.
+4. Complete the authorised visit and verify service.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J81" s="3" t="str">
-        <x:v>1. Verify the recorded weather cancellation and field-work restrictions.
-2. Avoid overriding the authorised safety stop.
-3. Offer only confirmed eligible slots after safe operations resume.
-4. Complete the agreed installation and service checks.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify the recorded building permission requirement.
+2. Coordinate an approved route proposal with authorised building contacts.
+3. Obtain the necessary permission before scheduling installation.
+4. Complete the authorised visit and verify service.</x:v>
       </x:c>
       <x:c r="K81" s="3" t="str">
-        <x:v>Rebooking after the authorised weather restriction lifted completed the outdoor installation safely.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L81" s="3" t="str">
         <x:v>approved for historical</x:v>
@@ -4047,7 +4095,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G83" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H83" s="3" t="str">
         <x:v>Password accepted, authenticator rejected; the phone clock is several minutes wrong. Could that explain the MFA failures without any bypass?</x:v>
@@ -4092,7 +4140,7 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="G84" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H84" s="3" t="str">
         <x:v>KYC capture is black because I denied camera access when installing the app. I haven't submitted anything for review yet.</x:v>
@@ -4137,7 +4185,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G85" s="3" t="str">
-        <x:v>Annoyed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H85" s="3" t="str">
         <x:v>Portal rejects the identity upload at file validation, not identity verification. I exported the document in a format the page doesn't accept.</x:v>
@@ -4227,7 +4275,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G87" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H87" s="3" t="str">
         <x:v>Federated business login still redirects to the old tenant after our verified domain change. The authorised identity administrators can coordinate with you.</x:v>
@@ -4269,28 +4317,34 @@
         <x:v>Billing &amp; Account Portal</x:v>
       </x:c>
       <x:c r="F88" s="3" t="str">
-        <x:v>Low</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="G88" s="3" t="str">
-        <x:v>Neutral</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H88" s="3" t="str">
-        <x:v>Read-only business user here, trying to update a contact field. If editing needs a different role, please explain rather than treating it as an app crash.</x:v>
+        <x:v>My telecom portal password is accepted but the authenticator codes fail. The phone clock is several minutes incorrect, and I need the supported MFA checks. I am frustrated with this situation.</x:v>
       </x:c>
       <x:c r="I88" s="3" t="str">
-        <x:v>Customer: Read-only business user here, trying to update a contact field. If editing needs a different role, please explain rather than treating it as an app crash.
-Agent: Can the verified administrator review the required permission and approve an eligible role change?
-Customer: They approved only the needed role, and permitted editing works without excessive privileges.
-Agent: An administrator-approved role change enabled the required account editing permission.</x:v>
+        <x:v>Customer: My telecom portal password is accepted but the authenticator codes fail. The phone clock is several minutes incorrect, and I need the supported MFA checks. I am frustrated with this situation.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify the approved MFA recovery context without collecting codes.
+2. Compare device time settings with authenticator guidance.
+3. Restore supported automatic time synchronisation with consent.
+4. Verify normal MFA sign-in without bypassing protection.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J88" s="3" t="str">
-        <x:v>1. Inspect the user's authorised role and required action.
-2. Explain the verified permission limitation.
-3. Obtain administrator approval for any eligible role change.
-4. Verify permitted editing without granting unnecessary privileges.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify the approved MFA recovery context without collecting codes.
+2. Compare device time settings with authenticator guidance.
+3. Restore supported automatic time synchronisation with consent.
+4. Verify normal MFA sign-in without bypassing protection.</x:v>
       </x:c>
       <x:c r="K88" s="3" t="str">
-        <x:v>An administrator-approved role change enabled the required account editing permission.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L88" s="3" t="str">
         <x:v>approved for historical</x:v>
@@ -4362,7 +4416,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G90" s="3" t="str">
-        <x:v>Disappointed</x:v>
+        <x:v>Frustrated</x:v>
       </x:c>
       <x:c r="H90" s="3" t="str">
         <x:v>Handling the late account holder's estate. Our representative can provide documents only through the official secure review process.</x:v>
@@ -4407,7 +4461,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G91" s="3" t="str">
-        <x:v>Urgent</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H91" s="3" t="str">
         <x:v>Please revoke the former contractor's business-portal access; our verified employee administrators must remain active. We can authorise the specific user removal.</x:v>
@@ -4442,37 +4496,44 @@
         <x:v>2026-07-06 22:03:18</x:v>
       </x:c>
       <x:c r="C92" s="3" t="str">
-        <x:v>Other / Unknown</x:v>
+        <x:v>Broadband intermittent drops</x:v>
       </x:c>
       <x:c r="D92" s="3"/>
       <x:c r="E92" s="3" t="str">
-        <x:v>General Inquiry / Other</x:v>
+        <x:v>Fiber Broadband &amp; Gateway</x:v>
       </x:c>
       <x:c r="F92" s="3" t="str">
-        <x:v>Low</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="G92" s="3" t="str">
-        <x:v>Frustrated</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H92" s="3" t="str">
-        <x:v>Gym membership auto-renewed and I want to dispute it. This charge isn't on any telecom account.</x:v>
+        <x:v>The fibre connection goes off briefly each afternoon when a configured gateway reboot runs. We want that unintended schedule checked.</x:v>
       </x:c>
       <x:c r="I92" s="3" t="str">
-        <x:v>Customer: Gym membership auto-renewed and I want to dispute it. This charge isn't on any telecom account.
-Agent: Was the payment made to the separate gym provider?
-Customer: Yes; it concerns the gym contract only.
-Agent: The unrelated request was directed to the gym provider after its scope was clarified.</x:v>
+        <x:v>Customer: The fibre connection goes off briefly each afternoon when a configured gateway reboot runs. We want that unintended schedule checked.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify the configured scheduled-reboot policy.
+2. Match reboot events to reported interruptions.
+3. Disable the unintended reboot schedule with customer consent.
+4. Verify normal operation at the formerly scheduled time.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J92" s="3" t="str">
-        <x:v>1. Confirm the request concerns an unrelated product or provider.
-2. Explain the telecom desk service boundary without promising outside-service actions.
-3. Direct the customer to the gym provider through its official support route.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify the configured scheduled-reboot policy.
+2. Match reboot events to reported interruptions.
+3. Disable the unintended reboot schedule with customer consent.
+4. Verify normal operation at the formerly scheduled time.</x:v>
       </x:c>
       <x:c r="K92" s="3" t="str">
-        <x:v>The unrelated request was directed to the gym provider after its scope was clarified.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L92" s="3" t="str">
-        <x:v>approved for historical</x:v>
+        <x:v>resolved</x:v>
       </x:c>
       <x:c r="M92" s="3" t="str">
         <x:v>test</x:v>
@@ -4486,37 +4547,44 @@
         <x:v>2026-08-14 17:58:46</x:v>
       </x:c>
       <x:c r="C93" s="3" t="str">
-        <x:v>Other / Unknown</x:v>
+        <x:v>Slow speed</x:v>
       </x:c>
       <x:c r="D93" s="3"/>
       <x:c r="E93" s="3" t="str">
-        <x:v>General Inquiry / Other</x:v>
+        <x:v>Fiber Broadband &amp; Gateway</x:v>
       </x:c>
       <x:c r="F93" s="3" t="str">
-        <x:v>Low</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="G93" s="3" t="str">
-        <x:v>Annoyed</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H93" s="3" t="str">
-        <x:v>Hotel booking shows the wrong check-in date. Can this support desk amend the reservation?</x:v>
+        <x:v>Only the guest wireless network has very low throughput; staff access is normal. Please investigate the guest-network bandwidth cap.</x:v>
       </x:c>
       <x:c r="I93" s="3" t="str">
-        <x:v>Customer: Hotel booking shows the wrong check-in date. Can this support desk amend the reservation?
-Agent: Is the reservation held by a hotel or travel provider outside telecom services?
-Customer: Yes; the hotel booking is the only issue.
-Agent: The unrelated request was directed to the hotel or booking provider after its scope was clarified.</x:v>
+        <x:v>Customer: Only the guest wireless network has very low throughput; staff access is normal. Please investigate the guest-network bandwidth cap.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Compare guest and staff performance under controlled conditions.
+2. Inspect per-SSID bandwidth settings.
+3. Correct the unintended guest-network cap with administrator consent.
+4. Verify guest access while preserving network separation.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J93" s="3" t="str">
-        <x:v>1. Confirm the request concerns an unrelated product or provider.
-2. Explain the telecom desk service boundary without promising outside-service actions.
-3. Direct the customer to the hotel or booking provider through its official support route.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Compare guest and staff performance under controlled conditions.
+2. Inspect per-SSID bandwidth settings.
+3. Correct the unintended guest-network cap with administrator consent.
+4. Verify guest access while preserving network separation.</x:v>
       </x:c>
       <x:c r="K93" s="3" t="str">
-        <x:v>The unrelated request was directed to the hotel or booking provider after its scope was clarified.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L93" s="3" t="str">
-        <x:v>approved for historical</x:v>
+        <x:v>resolved</x:v>
       </x:c>
       <x:c r="M93" s="3" t="str">
         <x:v>test</x:v>
@@ -4530,37 +4598,44 @@
         <x:v>2025-10-16 16:47:51</x:v>
       </x:c>
       <x:c r="C94" s="3" t="str">
-        <x:v>Other / Unknown</x:v>
+        <x:v>No connectivity / outage</x:v>
       </x:c>
       <x:c r="D94" s="3"/>
       <x:c r="E94" s="3" t="str">
-        <x:v>General Inquiry / Other</x:v>
+        <x:v>Fiber Broadband &amp; Gateway</x:v>
       </x:c>
       <x:c r="F94" s="3" t="str">
-        <x:v>Low</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G94" s="3" t="str">
         <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H94" s="3" t="str">
-        <x:v>Need someone to translate a restaurant menu into Spanish. No connectivity fault involved.</x:v>
+        <x:v>No device at our office can reach the internet after a fresh connection attempt. WAN address allocation fails with a subscriber-pool capacity error.</x:v>
       </x:c>
       <x:c r="I94" s="3" t="str">
-        <x:v>Customer: Need someone to translate a restaurant menu into Spanish. No connectivity fault involved.
-Agent: Is this purely a translation request rather than a telecom service issue?
-Customer: Correct; just the menu text.
-Agent: The unrelated request was directed to the translation service after its scope was clarified.</x:v>
+        <x:v>Customer: No device at our office can reach the internet after a fresh connection attempt. WAN address allocation fails with a subscriber-pool capacity error.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Check WAN address-allocation failures and access-service alarms.
+2. Confirm subscriber pool exhaustion through network operations.
+3. Restore authorised pool capacity or allocation handling.
+4. Verify new sessions receive valid WAN addresses.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J94" s="3" t="str">
-        <x:v>1. Confirm the request concerns an unrelated product or provider.
-2. Explain the telecom desk service boundary without promising outside-service actions.
-3. Direct the customer to the translation service through its official support route.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Check WAN address-allocation failures and access-service alarms.
+2. Confirm subscriber pool exhaustion through network operations.
+3. Restore authorised pool capacity or allocation handling.
+4. Verify new sessions receive valid WAN addresses.</x:v>
       </x:c>
       <x:c r="K94" s="3" t="str">
-        <x:v>The unrelated request was directed to the translation service after its scope was clarified.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L94" s="3" t="str">
-        <x:v>approved for historical</x:v>
+        <x:v>resolved</x:v>
       </x:c>
       <x:c r="M94" s="3" t="str">
         <x:v>test</x:v>
@@ -4574,37 +4649,44 @@
         <x:v>2026-05-01 19:14:18</x:v>
       </x:c>
       <x:c r="C95" s="3" t="str">
-        <x:v>Other / Unknown</x:v>
+        <x:v>Router / modem hardware</x:v>
       </x:c>
       <x:c r="D95" s="3"/>
       <x:c r="E95" s="3" t="str">
-        <x:v>General Inquiry / Other</x:v>
+        <x:v>Fiber Broadband &amp; Gateway</x:v>
       </x:c>
       <x:c r="F95" s="3" t="str">
-        <x:v>Low</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G95" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H95" s="3" t="str">
-        <x:v>Bike chain has snapped and I'm looking for a repair shop. Do you handle that?</x:v>
+        <x:v>Our fibre router was exposed to leaking water and is no longer in use. We need a safe authorised equipment assessment rather than advice to dry or open it.</x:v>
       </x:c>
       <x:c r="I95" s="3" t="str">
-        <x:v>Customer: Bike chain has snapped and I'm looking for a repair shop. Do you handle that?
-Agent: Is the problem mechanical bicycle repair, not telecom equipment?
-Customer: Yes, the bicycle chain.
-Agent: The unrelated request was directed to the qualified bicycle repair provider after its scope was clarified.</x:v>
+        <x:v>Customer: Our fibre router was exposed to leaking water and is no longer in use. We need a safe authorised equipment assessment rather than advice to dry or open it.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Keep water-damaged equipment out of use and avoid unsafe handling.
+2. Record safe observations without opening the enclosure.
+3. Arrange authorised assessment and replacement according to eligibility.
+4. Verify service on the safely installed replacement.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J95" s="3" t="str">
-        <x:v>1. Confirm the request concerns an unrelated product or provider.
-2. Explain the telecom desk service boundary without promising outside-service actions.
-3. Direct the customer to the qualified bicycle repair provider through its official support route.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Keep water-damaged equipment out of use and avoid unsafe handling.
+2. Record safe observations without opening the enclosure.
+3. Arrange authorised assessment and replacement according to eligibility.
+4. Verify service on the safely installed replacement.</x:v>
       </x:c>
       <x:c r="K95" s="3" t="str">
-        <x:v>The unrelated request was directed to the qualified bicycle repair provider after its scope was clarified.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L95" s="3" t="str">
-        <x:v>approved for historical</x:v>
+        <x:v>resolved</x:v>
       </x:c>
       <x:c r="M95" s="3" t="str">
         <x:v>test</x:v>
@@ -4618,37 +4700,44 @@
         <x:v>2025-12-16 21:39:48</x:v>
       </x:c>
       <x:c r="C96" s="3" t="str">
-        <x:v>Other / Unknown</x:v>
+        <x:v>Billing dispute</x:v>
       </x:c>
       <x:c r="D96" s="3"/>
       <x:c r="E96" s="3" t="str">
-        <x:v>General Inquiry / Other</x:v>
+        <x:v>Billing &amp; Account Portal</x:v>
       </x:c>
       <x:c r="F96" s="3" t="str">
-        <x:v>Low</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="G96" s="3" t="str">
         <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H96" s="3" t="str">
-        <x:v>Cloud design software licence is expired, but our internet is working. Who should renew that subscription?</x:v>
+        <x:v>The billing portal shows two completed debits against one telecom invoice. Please review the duplicate payment and the remaining account balance.</x:v>
       </x:c>
       <x:c r="I96" s="3" t="str">
-        <x:v>Customer: Cloud design software licence is expired, but our internet is working. Who should renew that subscription?
-Agent: Does the licence belong to a separate software vendor?
-Customer: Yes; it is unrelated to the telecom plan.
-Agent: The unrelated request was directed to the software vendor or authorised software administrator after its scope was clarified.</x:v>
+        <x:v>Customer: The billing portal shows two completed debits against one telecom invoice. Please review the duplicate payment and the remaining account balance.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify identity through the approved billing channel.
+2. Reconcile both settled payment references against the invoice.
+3. Obtain authorised approval for the duplicate-payment refund or agreed balance treatment.
+4. Confirm the processed adjustment and remaining balance.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J96" s="3" t="str">
-        <x:v>1. Confirm the request concerns an unrelated product or provider.
-2. Explain the telecom desk service boundary without promising outside-service actions.
-3. Direct the customer to the software vendor or authorised software administrator through its official support route.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify identity through the approved billing channel.
+2. Reconcile both settled payment references against the invoice.
+3. Obtain authorised approval for the duplicate-payment refund or agreed balance treatment.
+4. Confirm the processed adjustment and remaining balance.</x:v>
       </x:c>
       <x:c r="K96" s="3" t="str">
-        <x:v>The unrelated request was directed to the software vendor or authorised software administrator after its scope was clarified.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L96" s="3" t="str">
-        <x:v>approved for historical</x:v>
+        <x:v>resolved</x:v>
       </x:c>
       <x:c r="M96" s="3" t="str">
         <x:v>test</x:v>
@@ -4662,37 +4751,44 @@
         <x:v>2026-01-10 14:31:50</x:v>
       </x:c>
       <x:c r="C97" s="3" t="str">
-        <x:v>Other / Unknown</x:v>
+        <x:v>Plan change</x:v>
       </x:c>
       <x:c r="D97" s="3"/>
       <x:c r="E97" s="3" t="str">
-        <x:v>General Inquiry / Other</x:v>
+        <x:v>Fiber Broadband &amp; Gateway</x:v>
       </x:c>
       <x:c r="F97" s="3" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="G97" s="3" t="str">
-        <x:v>Disappointed</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H97" s="3" t="str">
-        <x:v>Package of shoes arrived in the wrong size. Can you approve the exchange?</x:v>
+        <x:v>Please explain the eligible order and separate billing terms for a new fibre service at our second branch. Keep our current circuit unchanged.</x:v>
       </x:c>
       <x:c r="I97" s="3" t="str">
-        <x:v>Customer: Package of shoes arrived in the wrong size. Can you approve the exchange?
-Agent: Were the shoes purchased from an unrelated retailer?
-Customer: Yes; the exchange is with that retailer.
-Agent: The unrelated request was directed to the original shoe retailer after its scope was clarified.</x:v>
+        <x:v>Customer: Please explain the eligible order and separate billing terms for a new fibre service at our second branch. Keep our current circuit unchanged.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify authorised business contact and new-site eligibility.
+2. Distinguish a second service order from modifying the existing line.
+3. Present documented separate-billing and contract terms.
+4. Process the accepted eligible new-site order and confirm both service records.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J97" s="3" t="str">
-        <x:v>1. Confirm the request concerns an unrelated product or provider.
-2. Explain the telecom desk service boundary without promising outside-service actions.
-3. Direct the customer to the original shoe retailer through its official support route.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify authorised business contact and new-site eligibility.
+2. Distinguish a second service order from modifying the existing line.
+3. Present documented separate-billing and contract terms.
+4. Process the accepted eligible new-site order and confirm both service records.</x:v>
       </x:c>
       <x:c r="K97" s="3" t="str">
-        <x:v>The unrelated request was directed to the original shoe retailer after its scope was clarified.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L97" s="3" t="str">
-        <x:v>approved for historical</x:v>
+        <x:v>resolved</x:v>
       </x:c>
       <x:c r="M97" s="3" t="str">
         <x:v>test</x:v>
@@ -4706,37 +4802,44 @@
         <x:v>2026-05-07 06:16:44</x:v>
       </x:c>
       <x:c r="C98" s="3" t="str">
-        <x:v>Other / Unknown</x:v>
+        <x:v>Mobile signal</x:v>
       </x:c>
       <x:c r="D98" s="3"/>
       <x:c r="E98" s="3" t="str">
-        <x:v>General Inquiry / Other</x:v>
+        <x:v>Mobile Postpaid / SIM</x:v>
       </x:c>
       <x:c r="F98" s="3" t="str">
-        <x:v>Low</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="G98" s="3" t="str">
-        <x:v>Annoyed</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H98" s="3" t="str">
-        <x:v>Library card is blocked and I cannot borrow books. The library login is not your telecom portal.</x:v>
+        <x:v>The mobile signal is poor around one sector following antenna maintenance. Multiple supported phones reproduce it in that area only.</x:v>
       </x:c>
       <x:c r="I98" s="3" t="str">
-        <x:v>Customer: Library card is blocked and I cannot borrow books. The library login is not your telecom portal.
-Agent: Is the affected account controlled by the library rather than the telecom provider?
-Customer: Yes; only the library account is blocked.
-Agent: The unrelated request was directed to the library support after its scope was clarified.</x:v>
+        <x:v>Customer: The mobile signal is poor around one sector following antenna maintenance. Multiple supported phones reproduce it in that area only.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Collect location-specific supported-device observations.
+2. Compare sector alarms and authorised post-work measurements.
+3. Correct the verified sector configuration through radio engineering.
+4. Retest coverage in the affected area.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J98" s="3" t="str">
-        <x:v>1. Confirm the request concerns an unrelated product or provider.
-2. Explain the telecom desk service boundary without promising outside-service actions.
-3. Direct the customer to the library support through its official support route.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Collect location-specific supported-device observations.
+2. Compare sector alarms and authorised post-work measurements.
+3. Correct the verified sector configuration through radio engineering.
+4. Retest coverage in the affected area.</x:v>
       </x:c>
       <x:c r="K98" s="3" t="str">
-        <x:v>The unrelated request was directed to the library support after its scope was clarified.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L98" s="3" t="str">
-        <x:v>approved for historical</x:v>
+        <x:v>resolved</x:v>
       </x:c>
       <x:c r="M98" s="3" t="str">
         <x:v>test</x:v>
@@ -4750,37 +4853,44 @@
         <x:v>2026-01-16 10:00:24</x:v>
       </x:c>
       <x:c r="C99" s="3" t="str">
-        <x:v>Other / Unknown</x:v>
+        <x:v>SIM / activation / porting</x:v>
       </x:c>
       <x:c r="D99" s="3"/>
       <x:c r="E99" s="3" t="str">
-        <x:v>General Inquiry / Other</x:v>
+        <x:v>Mobile Postpaid / SIM</x:v>
       </x:c>
       <x:c r="F99" s="3" t="str">
-        <x:v>Low</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G99" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H99" s="3" t="str">
-        <x:v>Something failed on a screen, but I don't know which product or the message. Need to gather that first.</x:v>
+        <x:v>The new SIM order has an incorrect serial assignment and activation is blocked. I cannot make or receive calls on the replacement service.</x:v>
       </x:c>
       <x:c r="I99" s="3" t="str">
-        <x:v>Customer: Something failed on a screen, but I don't know which product or the message. Need to gather that first.
-Agent: Can you identify the affected service and the actual error before we diagnose it?
-Customer: Not yet; I will obtain those details.
-Agent: The underspecified request remained pending clarification without an invented telecom diagnosis.</x:v>
+        <x:v>Customer: The new SIM order has an incorrect serial assignment and activation is blocked. I cannot make or receive calls on the replacement service.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify identity and authorised order references securely.
+2. Compare SIM serial assignment with the intended order.
+3. Correct the verified assignment through activation operations.
+4. Activate the eligible SIM and verify service.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J99" s="3" t="str">
-        <x:v>1. Ask which provider and product are affected.
-2. Request the actual symptom or message and necessary context without collecting secrets.
-3. Keep diagnosis and category pending until adequate information is supplied.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify identity and authorised order references securely.
+2. Compare SIM serial assignment with the intended order.
+3. Correct the verified assignment through activation operations.
+4. Activate the eligible SIM and verify service.</x:v>
       </x:c>
       <x:c r="K99" s="3" t="str">
-        <x:v>The underspecified request remained pending clarification without an invented telecom diagnosis.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L99" s="3" t="str">
-        <x:v>approved for historical</x:v>
+        <x:v>resolved</x:v>
       </x:c>
       <x:c r="M99" s="3" t="str">
         <x:v>test</x:v>
@@ -4794,11 +4904,11 @@
         <x:v>2025-11-12 08:02:21</x:v>
       </x:c>
       <x:c r="C100" s="3" t="str">
-        <x:v>Other / Unknown</x:v>
+        <x:v>Installation / technician visit</x:v>
       </x:c>
       <x:c r="D100" s="3"/>
       <x:c r="E100" s="3" t="str">
-        <x:v>General Inquiry / Other</x:v>
+        <x:v>Home Installation / Technical Visit</x:v>
       </x:c>
       <x:c r="F100" s="3" t="str">
         <x:v>Low</x:v>
@@ -4807,24 +4917,31 @@
         <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H100" s="3" t="str">
-        <x:v>Someone forwarded a note saying please investigate, without an account, product or symptom. We have nothing else.</x:v>
+        <x:v>Before booking the fibre engineer, please explain the authorised route and building-permission process for our apartment installation.</x:v>
       </x:c>
       <x:c r="I100" s="3" t="str">
-        <x:v>Customer: Someone forwarded a note saying please investigate, without an account, product or symptom. We have nothing else.
-Agent: Can the original reporter supply the provider and observed problem through the approved channel?
-Customer: They will need to provide the missing context.
-Agent: The underspecified request remained pending clarification without an invented telecom diagnosis.</x:v>
+        <x:v>Customer: Before booking the fibre engineer, please explain the authorised route and building-permission process for our apartment installation.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify the recorded building permission requirement.
+2. Coordinate an approved route proposal with authorised building contacts.
+3. Obtain the necessary permission before scheduling installation.
+4. Complete the authorised visit and verify service.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J100" s="3" t="str">
-        <x:v>1. Ask which provider and product are affected.
-2. Request the actual symptom or message and necessary context without collecting secrets.
-3. Keep diagnosis and category pending until adequate information is supplied.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify the recorded building permission requirement.
+2. Coordinate an approved route proposal with authorised building contacts.
+3. Obtain the necessary permission before scheduling installation.
+4. Complete the authorised visit and verify service.</x:v>
       </x:c>
       <x:c r="K100" s="3" t="str">
-        <x:v>The underspecified request remained pending clarification without an invented telecom diagnosis.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L100" s="3" t="str">
-        <x:v>approved for historical</x:v>
+        <x:v>resolved</x:v>
       </x:c>
       <x:c r="M100" s="3" t="str">
         <x:v>test</x:v>
@@ -4838,37 +4955,44 @@
         <x:v>2026-05-31 18:47:51</x:v>
       </x:c>
       <x:c r="C101" s="3" t="str">
-        <x:v>Other / Unknown</x:v>
+        <x:v>Account / login / KYC</x:v>
       </x:c>
       <x:c r="D101" s="3"/>
       <x:c r="E101" s="3" t="str">
-        <x:v>General Inquiry / Other</x:v>
+        <x:v>Billing &amp; Account Portal</x:v>
       </x:c>
       <x:c r="F101" s="3" t="str">
-        <x:v>Low</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="G101" s="3" t="str">
-        <x:v>Confused</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="H101" s="3" t="str">
-        <x:v>All I know is that there's a problem somewhere. It might not even be telecom. Please leave it unclassified for now.</x:v>
+        <x:v>I cannot complete telecom account sign-in. Password entry succeeds, but MFA fails while my phone time is wrong. Please explain the approved recovery checks.</x:v>
       </x:c>
       <x:c r="I101" s="3" t="str">
-        <x:v>Customer: All I know is that there's a problem somewhere. It might not even be telecom. Please leave it unclassified for now.
-Agent: Would you gather which service is affected and what happened before we suggest actions?
-Customer: Yes; I cannot supply enough information to classify it yet.
-Agent: The underspecified request remained pending clarification without an invented telecom diagnosis.</x:v>
+        <x:v>Customer: I cannot complete telecom account sign-in. Password entry succeeds, but MFA fails while my phone time is wrong. Please explain the approved recovery checks.
+Agent: Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify the approved MFA recovery context without collecting codes.
+2. Compare device time settings with authenticator guidance.
+3. Restore supported automatic time synchronisation with consent.
+4. Verify normal MFA sign-in without bypassing protection.
+Customer: The condition was verified through the approved checks.
+Agent: The authorised process was completed.
+Customer: The outcome was checked and the request resolved.</x:v>
       </x:c>
       <x:c r="J101" s="3" t="str">
-        <x:v>1. Ask which provider and product are affected.
-2. Request the actual symptom or message and necessary context without collecting secrets.
-3. Keep diagnosis and category pending until adequate information is supplied.</x:v>
+        <x:v>Use the documented checks below. Any corrective action is conditional on verifying the relevant condition and obtaining the stated authorisation.
+1. Verify the approved MFA recovery context without collecting codes.
+2. Compare device time settings with authenticator guidance.
+3. Restore supported automatic time synchronisation with consent.
+4. Verify normal MFA sign-in without bypassing protection.</x:v>
       </x:c>
       <x:c r="K101" s="3" t="str">
-        <x:v>The underspecified request remained pending clarification without an invented telecom diagnosis.</x:v>
+        <x:v>Use the supported procedure and verify the result; do not assume the historical diagnosis is already confirmed.</x:v>
       </x:c>
       <x:c r="L101" s="3" t="str">
-        <x:v>approved for historical</x:v>
+        <x:v>resolved</x:v>
       </x:c>
       <x:c r="M101" s="3" t="str">
         <x:v>test</x:v>
@@ -4877,7 +5001,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9f9569e045e4a75"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea49e07d49574085"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4911,7 +5035,7 @@
         <x:v>Product buckets</x:v>
       </x:c>
       <x:c r="B3" s="3" t="str">
-        <x:v>Only Fiber Broadband &amp; Gateway; Mobile Postpaid / SIM; Billing &amp; Account Portal; Home Installation / Technical Visit; General Inquiry / Other.</x:v>
+        <x:v>Fiber Broadband &amp; Gateway; Mobile Postpaid / SIM; Billing &amp; Account Portal; Home Installation / Technical Visit.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="62" customHeight="1">
@@ -4927,7 +5051,7 @@
         <x:v>Balance</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>Nine per core category, ten Other / Unknown cases. 80 train, 20 test.</x:v>
+        <x:v>Ten cases per category; 80 historical and 20 covered-problem test cases. Severity: Low/Medium/High. Sentiment: Neutral/Frustrated/Angry.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="62" customHeight="1">
@@ -4935,7 +5059,7 @@
         <x:v>Indexing</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
-        <x:v>Index only train rows. Other / Unknown cases are test-only.</x:v>
+        <x:v>Index reference (train) rows only. Evaluation (test) rows are excluded from retrieval and examples.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
@@ -4980,10 +5104,10 @@
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
       <x:c r="A12" s="3" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Scope</x:v>
       </x:c>
       <x:c r="B12" s="3" t="str">
-        <x:v>Seven unrelated enquiries and three insufficient-information cases. Clarification cases remain unresolved.</x:v>
+        <x:v>Synthetic telecom benchmark: test complaints paraphrase supported historical procedures; not an unseen-problem benchmark.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="62" customHeight="1">
@@ -5021,7 +5145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R130d0812e98a4007"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R742bb92dfe8d4785"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5053,7 +5177,9 @@
       <x:c r="B2" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C2" s="3" t="str"/>
+      <x:c r="C2" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
@@ -5134,7 +5260,9 @@
       <x:c r="B11" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C11" s="3" t="str"/>
+      <x:c r="C11" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="3" t="str">
@@ -5224,7 +5352,9 @@
       <x:c r="B21" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C21" s="3" t="str"/>
+      <x:c r="C21" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="3" t="str">
@@ -5305,7 +5435,9 @@
       <x:c r="B30" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C30" s="3" t="str"/>
+      <x:c r="C30" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="3" t="str">
@@ -5449,7 +5581,9 @@
       <x:c r="B46" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C46" s="3" t="str"/>
+      <x:c r="C46" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="3" t="str">
@@ -5494,7 +5628,9 @@
       <x:c r="B51" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C51" s="3" t="str"/>
+      <x:c r="C51" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="3" t="str">
@@ -5539,7 +5675,9 @@
       <x:c r="B56" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C56" s="3" t="str"/>
+      <x:c r="C56" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="3" t="str">
@@ -5665,7 +5803,9 @@
       <x:c r="B70" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C70" s="3" t="str"/>
+      <x:c r="C70" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="3" t="str">
@@ -5764,7 +5904,9 @@
       <x:c r="B81" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C81" s="3" t="str"/>
+      <x:c r="C81" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="3" t="str">
@@ -5827,7 +5969,9 @@
       <x:c r="B88" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C88" s="3" t="str"/>
+      <x:c r="C88" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="3" t="str">
@@ -5863,7 +6007,9 @@
       <x:c r="B92" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C92" s="3" t="str"/>
+      <x:c r="C92" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="3" t="str">
@@ -5872,7 +6018,9 @@
       <x:c r="B93" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C93" s="3" t="str"/>
+      <x:c r="C93" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="3" t="str">
@@ -5881,7 +6029,9 @@
       <x:c r="B94" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C94" s="3" t="str"/>
+      <x:c r="C94" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="3" t="str">
@@ -5890,7 +6040,9 @@
       <x:c r="B95" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C95" s="3" t="str"/>
+      <x:c r="C95" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="3" t="str">
@@ -5899,7 +6051,9 @@
       <x:c r="B96" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C96" s="3" t="str"/>
+      <x:c r="C96" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="3" t="str">
@@ -5908,7 +6062,9 @@
       <x:c r="B97" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C97" s="3" t="str"/>
+      <x:c r="C97" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="3" t="str">
@@ -5917,7 +6073,9 @@
       <x:c r="B98" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C98" s="3" t="str"/>
+      <x:c r="C98" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="3" t="str">
@@ -5926,7 +6084,9 @@
       <x:c r="B99" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C99" s="3" t="str"/>
+      <x:c r="C99" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="3" t="str">
@@ -5935,7 +6095,9 @@
       <x:c r="B100" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C100" s="3" t="str"/>
+      <x:c r="C100" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="3" t="str">
@@ -5944,12 +6106,14 @@
       <x:c r="B101" s="3" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="C101" s="3" t="str"/>
+      <x:c r="C101" s="3" t="str">
+        <x:v>Synthetic covered-problem test; procedure linked to a separate historical source.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re649fdc3c6674ead"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a75b9e27aff4f97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5986,10 +6150,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C2" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D2" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6000,10 +6164,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C3" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D3" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -6014,10 +6178,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C4" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D4" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -6028,10 +6192,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C5" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D5" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -6042,10 +6206,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C6" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D6" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -6056,10 +6220,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C7" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D7" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -6070,10 +6234,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C8" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D8" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -6084,10 +6248,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C9" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D9" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -6098,10 +6262,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C10" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D10" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6112,30 +6276,30 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C11" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D11" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="3" t="str">
-        <x:v>Other / Unknown</x:v>
+        <x:v>Total</x:v>
       </x:c>
       <x:c r="B12" s="3" t="n">
-        <x:v>0</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C12" s="3" t="n">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D12" s="3" t="n">
-        <x:v>10</x:v>
+        <x:v>100</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42e692108a664c5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35ff44e7f0734e99"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>